<commit_message>
HBM v0.4: recalibrate supply to broker output (UBS capacity, iM production), shared KGI demand with CoWoS; Minto pyramid layout; single reproducible build (build.sh, hbm/build.py, cowos/build.py); CoWoS v0.3 consistency; SOP v1.3 page spec
</commit_message>
<xml_diff>
--- a/cowos/cowos_model.xlsx
+++ b/cowos/cowos_model.xlsx
@@ -3124,57 +3124,57 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>单位：百万颗 AI 加速器封装/季；算法见 toc.js / data/toc.json；除 CoWoS、HBM 外各环节规模为估计（含校准）</t>
+          <t>单位：百万颗 AI 加速器封装/季；算法见 toc.js / data/toc.json；除 CoWoS、HBM 外各环节规模为估计（含校准）；由 cowos/build.py 生成</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>季度</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>需求</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>CoWoS</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>HBM</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>TC键合机</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>ABF载板</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="1" t="inlineStr">
         <is>
           <t>电力</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="1" t="inlineStr">
         <is>
           <t>最小环节</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="1" t="inlineStr">
         <is>
           <t>约束</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" s="1" t="inlineStr">
         <is>
           <t>通过量</t>
         </is>
@@ -3196,7 +3196,7 @@
         <v>1.47</v>
       </c>
       <c r="E3" t="n">
-        <v>2.524</v>
+        <v>3.274</v>
       </c>
       <c r="F3" t="n">
         <v>2.109</v>
@@ -3234,7 +3234,7 @@
         <v>1.79</v>
       </c>
       <c r="E4" t="n">
-        <v>3.158</v>
+        <v>4.097</v>
       </c>
       <c r="F4" t="n">
         <v>2.3</v>
@@ -3272,7 +3272,7 @@
         <v>2.749</v>
       </c>
       <c r="E5" t="n">
-        <v>3.793</v>
+        <v>4.92</v>
       </c>
       <c r="F5" t="n">
         <v>2.492</v>
@@ -3310,7 +3310,7 @@
         <v>3.58</v>
       </c>
       <c r="E6" t="n">
-        <v>4.427</v>
+        <v>5.743</v>
       </c>
       <c r="F6" t="n">
         <v>2.684</v>
@@ -3345,10 +3345,10 @@
         <v>2.331</v>
       </c>
       <c r="D7" t="n">
-        <v>2.603</v>
+        <v>3.377</v>
       </c>
       <c r="E7" t="n">
-        <v>2.863</v>
+        <v>3.714</v>
       </c>
       <c r="F7" t="n">
         <v>2.687</v>
@@ -3383,10 +3383,10 @@
         <v>2.961</v>
       </c>
       <c r="D8" t="n">
-        <v>2.744</v>
+        <v>3.678</v>
       </c>
       <c r="E8" t="n">
-        <v>3.434</v>
+        <v>4.455</v>
       </c>
       <c r="F8" t="n">
         <v>2.931</v>
@@ -3396,16 +3396,16 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>HBM</t>
+          <t>ABF 载板</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>HBM</t>
+          <t>需求（各环节都够）</t>
         </is>
       </c>
       <c r="J8" t="n">
-        <v>2.744</v>
+        <v>2.791</v>
       </c>
     </row>
     <row r="9">
@@ -3421,10 +3421,10 @@
         <v>3.591</v>
       </c>
       <c r="D9" t="n">
-        <v>2.886</v>
+        <v>3.978</v>
       </c>
       <c r="E9" t="n">
-        <v>4.005</v>
+        <v>5.196</v>
       </c>
       <c r="F9" t="n">
         <v>3.175</v>
@@ -3434,16 +3434,16 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>HBM</t>
+          <t>ABF 载板</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>HBM</t>
+          <t>需求（各环节都够）</t>
         </is>
       </c>
       <c r="J9" t="n">
-        <v>2.886</v>
+        <v>3.024</v>
       </c>
     </row>
     <row r="10">
@@ -3459,10 +3459,10 @@
         <v>4.221</v>
       </c>
       <c r="D10" t="n">
-        <v>3.03</v>
+        <v>4.281</v>
       </c>
       <c r="E10" t="n">
-        <v>4.576</v>
+        <v>5.937</v>
       </c>
       <c r="F10" t="n">
         <v>3.419</v>
@@ -3472,16 +3472,16 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>HBM</t>
+          <t>ABF 载板</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>HBM</t>
+          <t>需求（各环节都够）</t>
         </is>
       </c>
       <c r="J10" t="n">
-        <v>3.03</v>
+        <v>3.256</v>
       </c>
     </row>
     <row r="11">
@@ -3497,10 +3497,10 @@
         <v>4.457</v>
       </c>
       <c r="D11" t="n">
-        <v>3.424</v>
+        <v>5.141</v>
       </c>
       <c r="E11" t="n">
-        <v>5.608</v>
+        <v>7.275</v>
       </c>
       <c r="F11" t="n">
         <v>4.48</v>
@@ -3510,16 +3510,16 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>HBM</t>
+          <t>CoWoS</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>HBM</t>
+          <t>需求（各环节都够）</t>
         </is>
       </c>
       <c r="J11" t="n">
-        <v>3.424</v>
+        <v>4.349</v>
       </c>
     </row>
     <row r="12">
@@ -3535,10 +3535,10 @@
         <v>5.211</v>
       </c>
       <c r="D12" t="n">
-        <v>3.728</v>
+        <v>5.506</v>
       </c>
       <c r="E12" t="n">
-        <v>6.408</v>
+        <v>8.313000000000001</v>
       </c>
       <c r="F12" t="n">
         <v>4.887</v>
@@ -3548,16 +3548,16 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>HBM</t>
+          <t>ABF 载板</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>HBM</t>
+          <t>需求（各环节都够）</t>
         </is>
       </c>
       <c r="J12" t="n">
-        <v>3.728</v>
+        <v>4.745</v>
       </c>
     </row>
     <row r="13">
@@ -3573,10 +3573,10 @@
         <v>5.964</v>
       </c>
       <c r="D13" t="n">
-        <v>4.033</v>
+        <v>5.872</v>
       </c>
       <c r="E13" t="n">
-        <v>7.208</v>
+        <v>9.35</v>
       </c>
       <c r="F13" t="n">
         <v>5.294</v>
@@ -3586,16 +3586,16 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>HBM</t>
+          <t>ABF 载板</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>HBM</t>
+          <t>需求（各环节都够）</t>
         </is>
       </c>
       <c r="J13" t="n">
-        <v>4.033</v>
+        <v>5.14</v>
       </c>
     </row>
     <row r="14">
@@ -3611,10 +3611,10 @@
         <v>6.718</v>
       </c>
       <c r="D14" t="n">
-        <v>4.338</v>
+        <v>6.241</v>
       </c>
       <c r="E14" t="n">
-        <v>8.007999999999999</v>
+        <v>10.388</v>
       </c>
       <c r="F14" t="n">
         <v>5.701</v>
@@ -3624,16 +3624,16 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>HBM</t>
+          <t>ABF 载板</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>HBM</t>
+          <t>需求（各环节都够）</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>4.338</v>
+        <v>5.535</v>
       </c>
     </row>
     <row r="15">
@@ -3649,10 +3649,10 @@
         <v>7.346</v>
       </c>
       <c r="D15" t="n">
-        <v>4.726</v>
+        <v>7.428</v>
       </c>
       <c r="E15" t="n">
-        <v>10.085</v>
+        <v>13.083</v>
       </c>
       <c r="F15" t="n">
         <v>5.712</v>
@@ -3662,16 +3662,16 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>HBM</t>
+          <t>ABF 载板</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>HBM</t>
+          <t>ABF 载板</t>
         </is>
       </c>
       <c r="J15" t="n">
-        <v>4.726</v>
+        <v>5.712</v>
       </c>
     </row>
     <row r="16">
@@ -3687,10 +3687,10 @@
         <v>8.544</v>
       </c>
       <c r="D16" t="n">
-        <v>5.12</v>
+        <v>8.105</v>
       </c>
       <c r="E16" t="n">
-        <v>11.001</v>
+        <v>14.271</v>
       </c>
       <c r="F16" t="n">
         <v>6.231</v>
@@ -3700,16 +3700,16 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>HBM</t>
+          <t>ABF 载板</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>HBM</t>
+          <t>ABF 载板</t>
         </is>
       </c>
       <c r="J16" t="n">
-        <v>5.12</v>
+        <v>6.231</v>
       </c>
     </row>
     <row r="17">
@@ -3725,10 +3725,10 @@
         <v>9.742000000000001</v>
       </c>
       <c r="D17" t="n">
-        <v>5.515</v>
+        <v>8.782999999999999</v>
       </c>
       <c r="E17" t="n">
-        <v>11.917</v>
+        <v>15.459</v>
       </c>
       <c r="F17" t="n">
         <v>6.75</v>
@@ -3738,16 +3738,16 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>HBM</t>
+          <t>ABF 载板</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>HBM</t>
+          <t>ABF 载板</t>
         </is>
       </c>
       <c r="J17" t="n">
-        <v>5.515</v>
+        <v>6.75</v>
       </c>
     </row>
     <row r="18">
@@ -3763,10 +3763,10 @@
         <v>10.932</v>
       </c>
       <c r="D18" t="n">
-        <v>5.91</v>
+        <v>9.462</v>
       </c>
       <c r="E18" t="n">
-        <v>12.833</v>
+        <v>16.647</v>
       </c>
       <c r="F18" t="n">
         <v>7.269</v>
@@ -3776,16 +3776,16 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>HBM</t>
+          <t>ABF 载板</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>HBM</t>
+          <t>ABF 载板</t>
         </is>
       </c>
       <c r="J18" t="n">
-        <v>5.91</v>
+        <v>7.269</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
HBM v0.5: China ledger (parallel to global): domestic-accelerator HBM demand vs available (stockpile + gray + CXMT + XMC) 2024-27, China governing thought + 3 arguments, China blocks in base steps 3/4/5/7/8/12, C1-C7 predictions, CJ1-CJ4 falsification, A-share beneficiaries with evidence grades, sources 68-89; global ledger no longer counts CXMT (2027 HBM coverage 93% -> 90%); template supports cn ledger with build-time checks; SOP v1.5 two-ledger rule
</commit_message>
<xml_diff>
--- a/cowos/cowos_model.xlsx
+++ b/cowos/cowos_model.xlsx
@@ -3497,7 +3497,7 @@
         <v>4.457</v>
       </c>
       <c r="D11" t="n">
-        <v>5.141</v>
+        <v>5.11</v>
       </c>
       <c r="E11" t="n">
         <v>7.275</v>
@@ -3535,7 +3535,7 @@
         <v>5.211</v>
       </c>
       <c r="D12" t="n">
-        <v>5.506</v>
+        <v>5.445</v>
       </c>
       <c r="E12" t="n">
         <v>8.313000000000001</v>
@@ -3573,7 +3573,7 @@
         <v>5.964</v>
       </c>
       <c r="D13" t="n">
-        <v>5.872</v>
+        <v>5.781</v>
       </c>
       <c r="E13" t="n">
         <v>9.35</v>
@@ -3611,7 +3611,7 @@
         <v>6.718</v>
       </c>
       <c r="D14" t="n">
-        <v>6.241</v>
+        <v>6.118</v>
       </c>
       <c r="E14" t="n">
         <v>10.388</v>
@@ -3649,7 +3649,7 @@
         <v>7.346</v>
       </c>
       <c r="D15" t="n">
-        <v>7.428</v>
+        <v>7.245</v>
       </c>
       <c r="E15" t="n">
         <v>13.083</v>
@@ -3687,7 +3687,7 @@
         <v>8.544</v>
       </c>
       <c r="D16" t="n">
-        <v>8.105</v>
+        <v>7.874</v>
       </c>
       <c r="E16" t="n">
         <v>14.271</v>
@@ -3725,7 +3725,7 @@
         <v>9.742000000000001</v>
       </c>
       <c r="D17" t="n">
-        <v>8.782999999999999</v>
+        <v>8.502000000000001</v>
       </c>
       <c r="E17" t="n">
         <v>15.459</v>
@@ -3763,7 +3763,7 @@
         <v>10.932</v>
       </c>
       <c r="D18" t="n">
-        <v>9.462</v>
+        <v>9.131</v>
       </c>
       <c r="E18" t="n">
         <v>16.647</v>

</xml_diff>

<commit_message>
CoWoS v0.4.3: silicon interposer as its own TOC stage - 1 CoWoS-S wafer = 1 good interposer wafer, L/EFB bridges only; 2026 slack ~+20%, 2027 ~+3% (S-type only, not the binding stage; ABF still tightest); 2028 OK if demand <+23%; China: not a constraint. Fix 2027 AMD MI450/455 -> CoWoS-L, Venice -> EFB. Sources 65-78, falsify J6, preds C9-C10
</commit_message>
<xml_diff>
--- a/cowos/cowos_model.xlsx
+++ b/cowos/cowos_model.xlsx
@@ -12,8 +12,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="其他与供给" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="平衡表" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="季度产能" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TOC约束" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="硅中介层" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TOC约束" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2081,7 +2082,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>L</t>
         </is>
       </c>
       <c r="G38" s="2" t="n">
@@ -2123,7 +2124,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G39" s="2" t="n">
@@ -3097,14 +3098,316 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>见 cowos_chain.md 附录</t>
-        </is>
+          <t>v0.4.3：1 片 CoWoS-S 晶圆 = 1 片良品硅中介层晶圆；L/EFB 按每片 0.05 片硅桥折算；R 型不用硅。单位：千片 12 寸/年（需求、供给）与千片/月（年末产能）。估=自估</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>年份</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>S 型片数</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>S 型颗数(百万)</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>硅桥折算</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>其他(交换芯片)</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>中介层需求</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>年末产能(千片/月)</t>
+        </is>
+      </c>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>其中台积电</t>
+        </is>
+      </c>
+      <c r="I2" s="1" t="inlineStr">
+        <is>
+          <t>联电</t>
+        </is>
+      </c>
+      <c r="J2" s="1" t="inlineStr">
+        <is>
+          <t>其他/格罗方德</t>
+        </is>
+      </c>
+      <c r="K2" s="1" t="inlineStr">
+        <is>
+          <t>良品供给(千片/年)</t>
+        </is>
+      </c>
+      <c r="L2" s="1" t="inlineStr">
+        <is>
+          <t>余量%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B3" t="n">
+        <v>134</v>
+      </c>
+      <c r="C3" t="n">
+        <v>3.904</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>9</v>
+      </c>
+      <c r="F3" t="n">
+        <v>143</v>
+      </c>
+      <c r="G3" t="n">
+        <v>16</v>
+      </c>
+      <c r="H3" t="n">
+        <v>13</v>
+      </c>
+      <c r="I3" t="n">
+        <v>3</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>151.6</v>
+      </c>
+      <c r="L3" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B4" t="n">
+        <v>302.1</v>
+      </c>
+      <c r="C4" t="n">
+        <v>8.182</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="E4" t="n">
+        <v>18</v>
+      </c>
+      <c r="F4" t="n">
+        <v>322</v>
+      </c>
+      <c r="G4" t="n">
+        <v>41</v>
+      </c>
+      <c r="H4" t="n">
+        <v>35</v>
+      </c>
+      <c r="I4" t="n">
+        <v>6</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>326.7</v>
+      </c>
+      <c r="L4" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B5" t="n">
+        <v>318.7</v>
+      </c>
+      <c r="C5" t="n">
+        <v>6.842</v>
+      </c>
+      <c r="D5" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="E5" t="n">
+        <v>36</v>
+      </c>
+      <c r="F5" t="n">
+        <v>371.6</v>
+      </c>
+      <c r="G5" t="n">
+        <v>41</v>
+      </c>
+      <c r="H5" t="n">
+        <v>35</v>
+      </c>
+      <c r="I5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>453.4</v>
+      </c>
+      <c r="L5" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B6" t="n">
+        <v>390.1</v>
+      </c>
+      <c r="C6" t="n">
+        <v>7.207</v>
+      </c>
+      <c r="D6" t="n">
+        <v>34.9</v>
+      </c>
+      <c r="E6" t="n">
+        <v>54</v>
+      </c>
+      <c r="F6" t="n">
+        <v>479</v>
+      </c>
+      <c r="G6" t="n">
+        <v>61</v>
+      </c>
+      <c r="H6" t="n">
+        <v>55</v>
+      </c>
+      <c r="I6" t="n">
+        <v>6</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>573.2</v>
+      </c>
+      <c r="L6" t="n">
+        <v>19.7</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B7" t="n">
+        <v>617</v>
+      </c>
+      <c r="C7" t="n">
+        <v>10.854</v>
+      </c>
+      <c r="D7" t="n">
+        <v>75.90000000000001</v>
+      </c>
+      <c r="E7" t="n">
+        <v>90</v>
+      </c>
+      <c r="F7" t="n">
+        <v>783</v>
+      </c>
+      <c r="G7" t="n">
+        <v>83</v>
+      </c>
+      <c r="H7" t="n">
+        <v>75</v>
+      </c>
+      <c r="I7" t="n">
+        <v>6</v>
+      </c>
+      <c r="J7" t="n">
+        <v>2</v>
+      </c>
+      <c r="K7" t="n">
+        <v>806.3</v>
+      </c>
+      <c r="L7" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2028</v>
+      </c>
+      <c r="G8" t="n">
+        <v>91</v>
+      </c>
+      <c r="H8" t="n">
+        <v>75</v>
+      </c>
+      <c r="I8" t="n">
+        <v>6</v>
+      </c>
+      <c r="J8" t="n">
+        <v>10</v>
+      </c>
+      <c r="K8" t="n">
+        <v>965.7</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>台积电 2024/2025 年末自制（校准）</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2027 年台积电自制新增的盈亏平衡（千片/月）</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>16.1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2028 年中介层需求同比上限（%）</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>23.3</v>
       </c>
     </row>
   </sheetData>
@@ -3118,12 +3421,33 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J18"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>见 cowos_chain.md 附录</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
           <t>单位：百万颗 AI 加速器封装/季；算法见 toc.js / data/toc.json；除 CoWoS、HBM 外各环节规模为估计（含校准）；由 cowos/build.py 生成</t>
         </is>
       </c>
@@ -3146,35 +3470,40 @@
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
+          <t>硅中介层</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
           <t>HBM</t>
         </is>
       </c>
-      <c r="E2" s="1" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>TC键合机</t>
         </is>
       </c>
-      <c r="F2" s="1" t="inlineStr">
+      <c r="G2" s="1" t="inlineStr">
         <is>
           <t>ABF载板</t>
         </is>
       </c>
-      <c r="G2" s="1" t="inlineStr">
+      <c r="H2" s="1" t="inlineStr">
         <is>
           <t>电力</t>
         </is>
       </c>
-      <c r="H2" s="1" t="inlineStr">
+      <c r="I2" s="1" t="inlineStr">
         <is>
           <t>最小环节</t>
         </is>
       </c>
-      <c r="I2" s="1" t="inlineStr">
+      <c r="J2" s="1" t="inlineStr">
         <is>
           <t>约束</t>
         </is>
       </c>
-      <c r="J2" s="1" t="inlineStr">
+      <c r="K2" s="1" t="inlineStr">
         <is>
           <t>通过量</t>
         </is>
@@ -3193,28 +3522,31 @@
         <v>1.341</v>
       </c>
       <c r="D3" t="n">
+        <v>1.646</v>
+      </c>
+      <c r="E3" t="n">
         <v>1.47</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>3.274</v>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>2.109</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>2.517</v>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>CoWoS</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>CoWoS</t>
         </is>
       </c>
-      <c r="J3" t="n">
+      <c r="K3" t="n">
         <v>1.341</v>
       </c>
     </row>
@@ -3231,28 +3563,31 @@
         <v>1.779</v>
       </c>
       <c r="D4" t="n">
+        <v>2.127</v>
+      </c>
+      <c r="E4" t="n">
         <v>1.79</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>4.097</v>
       </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>2.3</v>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>2.517</v>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>CoWoS</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>CoWoS</t>
         </is>
       </c>
-      <c r="J4" t="n">
+      <c r="K4" t="n">
         <v>1.779</v>
       </c>
     </row>
@@ -3269,28 +3604,31 @@
         <v>2.217</v>
       </c>
       <c r="D5" t="n">
+        <v>2.609</v>
+      </c>
+      <c r="E5" t="n">
         <v>2.749</v>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>4.92</v>
       </c>
-      <c r="F5" t="n">
+      <c r="G5" t="n">
         <v>2.492</v>
       </c>
-      <c r="G5" t="n">
+      <c r="H5" t="n">
         <v>2.768</v>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>CoWoS</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>CoWoS</t>
         </is>
       </c>
-      <c r="J5" t="n">
+      <c r="K5" t="n">
         <v>2.217</v>
       </c>
     </row>
@@ -3307,28 +3645,31 @@
         <v>2.655</v>
       </c>
       <c r="D6" t="n">
+        <v>3.082</v>
+      </c>
+      <c r="E6" t="n">
         <v>3.58</v>
       </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
         <v>5.743</v>
       </c>
-      <c r="F6" t="n">
+      <c r="G6" t="n">
         <v>2.684</v>
       </c>
-      <c r="G6" t="n">
+      <c r="H6" t="n">
         <v>2.768</v>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>CoWoS</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>需求（各环节都够）</t>
         </is>
       </c>
-      <c r="J6" t="n">
+      <c r="K6" t="n">
         <v>2.44</v>
       </c>
     </row>
@@ -3345,28 +3686,31 @@
         <v>2.331</v>
       </c>
       <c r="D7" t="n">
+        <v>3.214</v>
+      </c>
+      <c r="E7" t="n">
         <v>3.377</v>
       </c>
-      <c r="E7" t="n">
+      <c r="F7" t="n">
         <v>3.714</v>
       </c>
-      <c r="F7" t="n">
+      <c r="G7" t="n">
         <v>2.687</v>
       </c>
-      <c r="G7" t="n">
+      <c r="H7" t="n">
         <v>3.07</v>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>CoWoS</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>CoWoS</t>
         </is>
       </c>
-      <c r="J7" t="n">
+      <c r="K7" t="n">
         <v>2.331</v>
       </c>
     </row>
@@ -3383,28 +3727,31 @@
         <v>2.961</v>
       </c>
       <c r="D8" t="n">
+        <v>3.302</v>
+      </c>
+      <c r="E8" t="n">
         <v>3.678</v>
       </c>
-      <c r="E8" t="n">
+      <c r="F8" t="n">
         <v>4.455</v>
       </c>
-      <c r="F8" t="n">
+      <c r="G8" t="n">
         <v>2.931</v>
       </c>
-      <c r="G8" t="n">
+      <c r="H8" t="n">
         <v>3.07</v>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>ABF 载板</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>需求（各环节都够）</t>
         </is>
       </c>
-      <c r="J8" t="n">
+      <c r="K8" t="n">
         <v>2.791</v>
       </c>
     </row>
@@ -3421,28 +3768,31 @@
         <v>3.591</v>
       </c>
       <c r="D9" t="n">
+        <v>3.391</v>
+      </c>
+      <c r="E9" t="n">
         <v>3.978</v>
       </c>
-      <c r="E9" t="n">
+      <c r="F9" t="n">
         <v>5.196</v>
       </c>
-      <c r="F9" t="n">
+      <c r="G9" t="n">
         <v>3.175</v>
       </c>
-      <c r="G9" t="n">
+      <c r="H9" t="n">
         <v>3.93</v>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>ABF 载板</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>需求（各环节都够）</t>
         </is>
       </c>
-      <c r="J9" t="n">
+      <c r="K9" t="n">
         <v>3.024</v>
       </c>
     </row>
@@ -3459,28 +3809,31 @@
         <v>4.221</v>
       </c>
       <c r="D10" t="n">
+        <v>3.479</v>
+      </c>
+      <c r="E10" t="n">
         <v>4.281</v>
       </c>
-      <c r="E10" t="n">
+      <c r="F10" t="n">
         <v>5.937</v>
       </c>
-      <c r="F10" t="n">
+      <c r="G10" t="n">
         <v>3.419</v>
       </c>
-      <c r="G10" t="n">
+      <c r="H10" t="n">
         <v>3.93</v>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>ABF 载板</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>需求（各环节都够）</t>
         </is>
       </c>
-      <c r="J10" t="n">
+      <c r="K10" t="n">
         <v>3.256</v>
       </c>
     </row>
@@ -3497,28 +3850,31 @@
         <v>4.457</v>
       </c>
       <c r="D11" t="n">
+        <v>4.722</v>
+      </c>
+      <c r="E11" t="n">
         <v>5.11</v>
       </c>
-      <c r="E11" t="n">
+      <c r="F11" t="n">
         <v>7.275</v>
       </c>
-      <c r="F11" t="n">
+      <c r="G11" t="n">
         <v>4.48</v>
       </c>
-      <c r="G11" t="n">
+      <c r="H11" t="n">
         <v>6.755</v>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>CoWoS</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>需求（各环节都够）</t>
         </is>
       </c>
-      <c r="J11" t="n">
+      <c r="K11" t="n">
         <v>4.349</v>
       </c>
     </row>
@@ -3535,28 +3891,31 @@
         <v>5.211</v>
       </c>
       <c r="D12" t="n">
+        <v>5.215</v>
+      </c>
+      <c r="E12" t="n">
         <v>5.445</v>
       </c>
-      <c r="E12" t="n">
+      <c r="F12" t="n">
         <v>8.313000000000001</v>
       </c>
-      <c r="F12" t="n">
+      <c r="G12" t="n">
         <v>4.887</v>
       </c>
-      <c r="G12" t="n">
+      <c r="H12" t="n">
         <v>6.755</v>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>ABF 载板</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>需求（各环节都够）</t>
         </is>
       </c>
-      <c r="J12" t="n">
+      <c r="K12" t="n">
         <v>4.745</v>
       </c>
     </row>
@@ -3573,28 +3932,31 @@
         <v>5.964</v>
       </c>
       <c r="D13" t="n">
+        <v>5.709</v>
+      </c>
+      <c r="E13" t="n">
         <v>5.781</v>
       </c>
-      <c r="E13" t="n">
+      <c r="F13" t="n">
         <v>9.35</v>
       </c>
-      <c r="F13" t="n">
+      <c r="G13" t="n">
         <v>5.294</v>
       </c>
-      <c r="G13" t="n">
+      <c r="H13" t="n">
         <v>7.025</v>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>ABF 载板</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>需求（各环节都够）</t>
         </is>
       </c>
-      <c r="J13" t="n">
+      <c r="K13" t="n">
         <v>5.14</v>
       </c>
     </row>
@@ -3611,28 +3973,31 @@
         <v>6.718</v>
       </c>
       <c r="D14" t="n">
+        <v>6.203</v>
+      </c>
+      <c r="E14" t="n">
         <v>6.118</v>
       </c>
-      <c r="E14" t="n">
+      <c r="F14" t="n">
         <v>10.388</v>
       </c>
-      <c r="F14" t="n">
+      <c r="G14" t="n">
         <v>5.701</v>
       </c>
-      <c r="G14" t="n">
+      <c r="H14" t="n">
         <v>7.025</v>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>ABF 载板</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>需求（各环节都够）</t>
         </is>
       </c>
-      <c r="J14" t="n">
+      <c r="K14" t="n">
         <v>5.535</v>
       </c>
     </row>
@@ -3649,28 +4014,31 @@
         <v>7.346</v>
       </c>
       <c r="D15" t="n">
+        <v>8.186999999999999</v>
+      </c>
+      <c r="E15" t="n">
         <v>7.245</v>
       </c>
-      <c r="E15" t="n">
+      <c r="F15" t="n">
         <v>13.083</v>
       </c>
-      <c r="F15" t="n">
+      <c r="G15" t="n">
         <v>5.712</v>
       </c>
-      <c r="G15" t="n">
+      <c r="H15" t="n">
         <v>10.126</v>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>ABF 载板</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>ABF 载板</t>
         </is>
       </c>
-      <c r="J15" t="n">
+      <c r="K15" t="n">
         <v>5.712</v>
       </c>
     </row>
@@ -3687,28 +4055,31 @@
         <v>8.544</v>
       </c>
       <c r="D16" t="n">
+        <v>8.94</v>
+      </c>
+      <c r="E16" t="n">
         <v>7.874</v>
       </c>
-      <c r="E16" t="n">
+      <c r="F16" t="n">
         <v>14.271</v>
       </c>
-      <c r="F16" t="n">
+      <c r="G16" t="n">
         <v>6.231</v>
       </c>
-      <c r="G16" t="n">
+      <c r="H16" t="n">
         <v>10.126</v>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>ABF 载板</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="J16" t="inlineStr">
         <is>
           <t>ABF 载板</t>
         </is>
       </c>
-      <c r="J16" t="n">
+      <c r="K16" t="n">
         <v>6.231</v>
       </c>
     </row>
@@ -3725,28 +4096,31 @@
         <v>9.742000000000001</v>
       </c>
       <c r="D17" t="n">
+        <v>9.694000000000001</v>
+      </c>
+      <c r="E17" t="n">
         <v>8.502000000000001</v>
       </c>
-      <c r="E17" t="n">
+      <c r="F17" t="n">
         <v>15.459</v>
       </c>
-      <c r="F17" t="n">
+      <c r="G17" t="n">
         <v>6.75</v>
       </c>
-      <c r="G17" t="n">
+      <c r="H17" t="n">
         <v>10.126</v>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="I17" t="inlineStr">
         <is>
           <t>ABF 载板</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="J17" t="inlineStr">
         <is>
           <t>ABF 载板</t>
         </is>
       </c>
-      <c r="J17" t="n">
+      <c r="K17" t="n">
         <v>6.75</v>
       </c>
     </row>
@@ -3763,28 +4137,31 @@
         <v>10.932</v>
       </c>
       <c r="D18" t="n">
+        <v>10.448</v>
+      </c>
+      <c r="E18" t="n">
         <v>9.131</v>
       </c>
-      <c r="E18" t="n">
+      <c r="F18" t="n">
         <v>16.647</v>
       </c>
-      <c r="F18" t="n">
+      <c r="G18" t="n">
         <v>7.269</v>
       </c>
-      <c r="G18" t="n">
+      <c r="H18" t="n">
         <v>10.126</v>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>ABF 载板</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>ABF 载板</t>
         </is>
       </c>
-      <c r="J18" t="n">
+      <c r="K18" t="n">
         <v>7.269</v>
       </c>
     </row>

</xml_diff>